<commit_message>
atualizaçao da lógica para apontamentos (fabrica em geral)
</commit_message>
<xml_diff>
--- a/utils/Modelos Importação/preenchido/Importar_Familia 2025-8-13.xlsx
+++ b/utils/Modelos Importação/preenchido/Importar_Familia 2025-8-13.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Odeclei\Projeto James\01 - Teste Apontamento Produção\Apontamento Produção 4.0\utils\Modelos Importação\preenchido\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projeto James\01 - Teste Apontamento Produção\Erp-4.0.0\utils\Modelos Importação\preenchido\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD6D8B3-210F-4A57-9BAA-1C68A9021D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D95143D-9A31-4F21-A0C0-FC27F1CBC1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="27510" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tablib Dataset" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
@@ -28,9 +28,6 @@
     <t>refer</t>
   </si>
   <si>
-    <t>description</t>
-  </si>
-  <si>
     <t>1054</t>
   </si>
   <si>
@@ -548,13 +545,16 @@
   </si>
   <si>
     <t>SOHO</t>
+  </si>
+  <si>
+    <t>name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -566,6 +566,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -588,9 +594,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -908,8 +915,8 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
+      <c r="C1" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -917,10 +924,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -928,10 +935,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -939,10 +946,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -950,10 +957,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -961,10 +968,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -972,10 +979,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -983,10 +990,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -994,10 +1001,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1005,10 +1012,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1016,10 +1023,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1027,10 +1034,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1038,10 +1045,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1049,10 +1056,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1060,10 +1067,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1071,10 +1078,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1082,10 +1089,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1093,10 +1100,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1104,10 +1111,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1115,10 +1122,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1126,10 +1133,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1137,10 +1144,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1148,10 +1155,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1159,10 +1166,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1170,10 +1177,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1181,10 +1188,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1192,10 +1199,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1203,10 +1210,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1214,10 +1221,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1225,10 +1232,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C30" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1236,10 +1243,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1247,10 +1254,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1258,10 +1265,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1269,10 +1276,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C34" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1280,10 +1287,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C35" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1291,10 +1298,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1302,10 +1309,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1313,10 +1320,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1324,10 +1331,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1335,10 +1342,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1346,10 +1353,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1357,10 +1364,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C42" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1368,10 +1375,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1379,10 +1386,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C44" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1390,10 +1397,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C45" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1401,10 +1408,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C46" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1412,10 +1419,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1423,10 +1430,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C48" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1434,10 +1441,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C49" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1445,10 +1452,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C50" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1456,10 +1463,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C51" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1467,10 +1474,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C52" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1478,10 +1485,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C53" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1489,10 +1496,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C54" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1500,10 +1507,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -1511,10 +1518,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C56" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1522,10 +1529,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C57" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1533,10 +1540,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C58" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1544,10 +1551,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1555,10 +1562,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C60" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1566,10 +1573,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C61" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1577,10 +1584,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C62" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1588,10 +1595,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C63" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1599,10 +1606,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C64" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -1610,10 +1617,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C65" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -1621,10 +1628,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C66" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -1632,10 +1639,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C67" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -1643,10 +1650,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C68" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -1654,10 +1661,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -1665,10 +1672,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C70" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -1676,10 +1683,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C71" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -1687,10 +1694,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C72" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -1698,10 +1705,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C73" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -1709,10 +1716,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1720,10 +1727,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C75" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1731,10 +1738,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C76" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1742,10 +1749,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C77" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1753,10 +1760,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C78" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1764,10 +1771,10 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C79" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1775,10 +1782,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1786,10 +1793,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C81" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -1797,10 +1804,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C82" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -1808,10 +1815,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C83" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1819,10 +1826,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C84" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1830,10 +1837,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C85" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1841,10 +1848,10 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C86" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1852,10 +1859,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C87" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1863,10 +1870,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C88" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>